<commit_message>
feat(financeiro): adicionar campo data de pagamento no modelo e sincronizar com vencimento quando nao preenchido
</commit_message>
<xml_diff>
--- a/public/modelos/Contas_a_Receber.xlsx
+++ b/public/modelos/Contas_a_Receber.xlsx
@@ -397,16 +397,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:I4"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
-    <col min="2" max="2" width="20.83203125" customWidth="1"/>
+    <col min="2" max="2" width="22.83203125" customWidth="1"/>
     <col min="3" max="3" width="15.83203125" customWidth="1"/>
     <col min="4" max="4" width="15.83203125" customWidth="1"/>
-    <col min="5" max="5" width="22.83203125" customWidth="1"/>
+    <col min="5" max="5" width="20.83203125" customWidth="1"/>
     <col min="6" max="6" width="22.83203125" customWidth="1"/>
-    <col min="7" max="7" width="28.83203125" customWidth="1"/>
-    <col min="8" max="8" width="15.83203125" customWidth="1"/>
+    <col min="7" max="7" width="20.83203125" customWidth="1"/>
+    <col min="8" max="8" width="28.83203125" customWidth="1"/>
+    <col min="9" max="9" width="15.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -423,15 +424,18 @@
         <v>Vencimento</v>
       </c>
       <c r="E1" t="str">
+        <v>Data de Pagamento</v>
+      </c>
+      <c r="F1" t="str">
         <v>Forma de Pagamento</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Caixa / Origem</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Cliente</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>Status</v>
       </c>
     </row>
@@ -440,7 +444,7 @@
         <v>Consultoria Técnica</v>
       </c>
       <c r="B2" t="str">
-        <v>Serviços</v>
+        <v>Prestação de Serviços</v>
       </c>
       <c r="C2">
         <v>1500</v>
@@ -449,16 +453,19 @@
         <v>20/10/2026</v>
       </c>
       <c r="E2" t="str">
+        <v>20/10/2026</v>
+      </c>
+      <c r="F2" t="str">
         <v>Pix</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
         <v>Caixa Principal</v>
       </c>
-      <c r="G2" t="str">
+      <c r="H2" t="str">
         <v>Empresa Exemplo LTDA</v>
       </c>
-      <c r="H2" t="str">
-        <v>Pendente</v>
+      <c r="I2" t="str">
+        <v>Recebido</v>
       </c>
     </row>
     <row r="3">
@@ -475,15 +482,18 @@
         <v>25/10/2026</v>
       </c>
       <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
         <v>Boleto</v>
       </c>
-      <c r="F3" t="str">
+      <c r="G3" t="str">
         <v>Conta Bancária</v>
       </c>
-      <c r="G3" t="str">
+      <c r="H3" t="str">
         <v/>
       </c>
-      <c r="H3" t="str">
+      <c r="I3" t="str">
         <v>Pendente</v>
       </c>
     </row>
@@ -492,7 +502,7 @@
         <v>Manutenção Preventiva</v>
       </c>
       <c r="B4" t="str">
-        <v>Serviços</v>
+        <v>Prestação de Serviços</v>
       </c>
       <c r="C4">
         <v>420</v>
@@ -501,21 +511,24 @@
         <v>15/10/2026</v>
       </c>
       <c r="E4" t="str">
+        <v>14/10/2026</v>
+      </c>
+      <c r="F4" t="str">
         <v>Cartão de Crédito</v>
       </c>
-      <c r="F4" t="str">
+      <c r="G4" t="str">
         <v>Caixa Principal</v>
       </c>
-      <c r="G4" t="str">
+      <c r="H4" t="str">
         <v>João da Silva</v>
       </c>
-      <c r="H4" t="str">
+      <c r="I4" t="str">
         <v>Recebido</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>